<commit_message>
Fix error allergy code (#105)
* Update FRAllergyIntoleranceDocument profile

* Update FRAllergyIntoleranceDocument profile
Co-authored-by: Nom Prenom <email@exemple.com>

* update FRAllergyIntoleranceDocument Profile

Co-authored-by: Troudi Haoura <haoura.troudi.ext@esante.gouv.fr>

---------

Co-authored-by: Troudi Haoura <haoura.troudi.ext@esante.gouv.fr> 6af81e3751dc88a352c1ae6f88a7e059c367753e
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-allergie-intolerance-document.xlsx
+++ b/main/ig/StructureDefinition-fr-allergie-intolerance-document.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="353">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-30T15:11:58+00:00</t>
+    <t>2026-03-31T07:16:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -555,7 +555,7 @@
 Class</t>
   </si>
   <si>
-    <t>allergy | intolerance - Underlying mechanism (if known)</t>
+    <t>Type d'allergie ou d'intolérance</t>
   </si>
   <si>
     <t>Identification of the underlying physiological mechanism for the reaction risk.</t>
@@ -564,10 +564,7 @@
     <t>Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
   </si>
   <si>
-    <t>Identification of the underlying physiological mechanism for a Reaction Risk.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/allergy-intolerance-type|4.0.1</t>
+    <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-vs-allergy-intolerance-type-document</t>
   </si>
   <si>
     <t>code</t>
@@ -645,7 +642,7 @@
 </t>
   </si>
   <si>
-    <t>Type d'allergie / hypersensibilité non allergique / intolérance / idiosyncrasie</t>
+    <t>agent allergique</t>
   </si>
   <si>
     <t>Code for an allergy or intolerance statement (either a positive or a negated/excluded statement).  This may be a code for a substance or pharmaceutical product that is considered to be responsible for the adverse reaction risk (e.g., "Latex"), an allergy or intolerance condition (e.g., "Latex allergy"), or a negated/excluded code for a specific substance or class (e.g., "No latex allergy") or a general or categorical negated statement (e.g.,  "No known allergy", "No known drug allergies").  Note: the substance for a specific reaction may be different from the substance identified as the cause of the risk, but it must be consistent with it. For instance, it may be a more specific substance (e.g. a brand medication) or a composite product that includes the identified substance. It must be clinically safe to only process the 'code' and ignore the 'reaction.substance'.  If a receiving system is unable to confirm that AllergyIntolerance.reaction.substance falls within the semantic scope of AllergyIntolerance.code, then the receiving system should ignore AllergyIntolerance.reaction.substance.</t>
@@ -658,7 +655,10 @@
 The 'substanceExposureRisk' extension is available as a structured and more flexible alternative to the 'code' element for making positive or negative allergy or intolerance statements.  This extension provides the capability to make "no known allergy" (or "no risk of adverse reaction") statements regarding any coded substance/product (including cases when a pre-coordinated "no allergy to x" concept for that substance/product does not exist).  If the 'substanceExposureRisk' extension is present, the AllergyIntolerance.code element SHALL be omitted.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-type-evenement-indesirable-previsible-cisis</t>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-vs-allergy-code</t>
   </si>
   <si>
     <t>substance/product:@@ -1010,16 +1010,13 @@
     <t>AllergyIntolerance.reaction.substance</t>
   </si>
   <si>
-    <t>Agent responsable de l'allergie / intolérance</t>
+    <t>Substance responsable de la réaction</t>
   </si>
   <si>
     <t>Identification of the specific substance (or pharmaceutical product) considered to be responsible for the Adverse Reaction event. Note: the substance for a specific reaction may be different from the substance identified as the cause of the risk, but it must be consistent with it. For instance, it may be a more specific substance (e.g. a brand medication) or a composite product that includes the identified substance. It must be clinically safe to only process the 'code' and ignore the 'reaction.substance'.  If a receiving system is unable to confirm that AllergyIntolerance.reaction.substance falls within the semantic scope of AllergyIntolerance.code, then the receiving system should ignore AllergyIntolerance.reaction.substance.</t>
   </si>
   <si>
     <t>Coding of the specific substance (or pharmaceutical product) with a terminology capable of triggering decision support should be used wherever possible.  The 'code' element allows for the use of a specific substance or pharmaceutical product, or a group or class of substances. In the case of an allergy or intolerance to a class of substances, (for example, "penicillins"), the 'reaction.substance' element could be used to code the specific substance that was identified as having caused the reaction (for example, "amoxycillin"). Duplication of the value in the 'code' and 'reaction.substance' elements is acceptable when a specific substance has been recorded in 'code'.</t>
-  </si>
-  <si>
-    <t>extensible</t>
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-vs-allergy-substance</t>
@@ -1480,7 +1477,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="106.67578125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="69.97265625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="77.98828125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -2948,7 +2945,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" hidden="true">
+    <row r="14">
       <c r="A14" t="s" s="2">
         <v>170</v>
       </c>
@@ -2967,7 +2964,7 @@
         <v>87</v>
       </c>
       <c r="H14" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I14" t="s" s="2">
         <v>79</v>
@@ -3013,11 +3010,9 @@
       <c r="X14" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="Y14" t="s" s="2">
+      <c r="Y14" s="2"/>
+      <c r="Z14" t="s" s="2">
         <v>175</v>
-      </c>
-      <c r="Z14" t="s" s="2">
-        <v>176</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>79</v>
@@ -3050,25 +3045,25 @@
         <v>99</v>
       </c>
       <c r="AK14" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="AL14" t="s" s="2">
         <v>177</v>
       </c>
-      <c r="AL14" t="s" s="2">
+      <c r="AM14" t="s" s="2">
         <v>178</v>
-      </c>
-      <c r="AM14" t="s" s="2">
-        <v>179</v>
       </c>
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
@@ -3090,13 +3085,13 @@
         <v>107</v>
       </c>
       <c r="L15" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="M15" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="M15" t="s" s="2">
+      <c r="N15" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>184</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
@@ -3125,11 +3120,11 @@
         <v>158</v>
       </c>
       <c r="Y15" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="Z15" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="Z15" t="s" s="2">
-        <v>186</v>
-      </c>
       <c r="AA15" t="s" s="2">
         <v>79</v>
       </c>
@@ -3146,7 +3141,7 @@
         <v>79</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>77</v>
@@ -3161,25 +3156,25 @@
         <v>99</v>
       </c>
       <c r="AK15" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AM15" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
@@ -3201,13 +3196,13 @@
         <v>107</v>
       </c>
       <c r="L16" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="M16" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="M16" t="s" s="2">
+      <c r="N16" t="s" s="2">
         <v>192</v>
-      </c>
-      <c r="N16" t="s" s="2">
-        <v>193</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
@@ -3236,11 +3231,11 @@
         <v>158</v>
       </c>
       <c r="Y16" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="Z16" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Z16" t="s" s="2">
-        <v>195</v>
-      </c>
       <c r="AA16" t="s" s="2">
         <v>79</v>
       </c>
@@ -3257,7 +3252,7 @@
         <v>79</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
@@ -3272,25 +3267,25 @@
         <v>99</v>
       </c>
       <c r="AK16" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="AL16" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="AL16" t="s" s="2">
+      <c r="AM16" t="s" s="2">
         <v>197</v>
-      </c>
-      <c r="AM16" t="s" s="2">
-        <v>198</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
@@ -3312,13 +3307,13 @@
         <v>154</v>
       </c>
       <c r="L17" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="M17" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="N17" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3344,7 +3339,7 @@
         <v>79</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="Y17" s="2"/>
       <c r="Z17" t="s" s="2">
@@ -3366,7 +3361,7 @@
         <v>79</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
@@ -5326,11 +5321,11 @@
         <v>79</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>315</v>
+        <v>158</v>
       </c>
       <c r="Y35" s="2"/>
       <c r="Z35" t="s" s="2">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>79</v>
@@ -5363,7 +5358,7 @@
         <v>99</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>79</v>
@@ -5374,14 +5369,14 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -5403,13 +5398,13 @@
         <v>154</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>321</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>322</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -5435,14 +5430,14 @@
         <v>79</v>
       </c>
       <c r="X36" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="Y36" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="Y36" t="s" s="2">
+      <c r="Z36" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="Z36" t="s" s="2">
-        <v>325</v>
-      </c>
       <c r="AA36" t="s" s="2">
         <v>79</v>
       </c>
@@ -5459,7 +5454,7 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>87</v>
@@ -5474,25 +5469,25 @@
         <v>99</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5514,13 +5509,13 @@
         <v>236</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>329</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>330</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>331</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5570,7 +5565,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
@@ -5585,7 +5580,7 @@
         <v>99</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
@@ -5596,10 +5591,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5625,10 +5620,10 @@
         <v>249</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>334</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>335</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5679,7 +5674,7 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
@@ -5700,15 +5695,15 @@
         <v>79</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5734,13 +5729,13 @@
         <v>107</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="N39" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -5769,11 +5764,11 @@
         <v>158</v>
       </c>
       <c r="Y39" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="Z39" t="s" s="2">
         <v>341</v>
       </c>
-      <c r="Z39" t="s" s="2">
-        <v>342</v>
-      </c>
       <c r="AA39" t="s" s="2">
         <v>79</v>
       </c>
@@ -5790,7 +5785,7 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
@@ -5805,7 +5800,7 @@
         <v>99</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>79</v>
@@ -5816,10 +5811,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5845,13 +5840,13 @@
         <v>154</v>
       </c>
       <c r="L40" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="M40" t="s" s="2">
+      <c r="N40" t="s" s="2">
         <v>345</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>346</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -5877,14 +5872,14 @@
         <v>79</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Y40" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="Z40" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="Z40" t="s" s="2">
-        <v>348</v>
-      </c>
       <c r="AA40" t="s" s="2">
         <v>79</v>
       </c>
@@ -5901,7 +5896,7 @@
         <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
@@ -5916,7 +5911,7 @@
         <v>99</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>79</v>
@@ -5927,10 +5922,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5956,13 +5951,13 @@
         <v>294</v>
       </c>
       <c r="L41" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="M41" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="M41" t="s" s="2">
+      <c r="N41" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>353</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -6012,7 +6007,7 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>

</xml_diff>